<commit_message>
review lenses: day in the life, operating rhythm, scenario walkthroughs
Persona registry (scripts/personas.py; overlay personas[] override) with
#/persona/<key> blueprint pages (moments x what you do / hand-offs / where /
what changes, flow diagrams dimmed to the role's steps, role gap list);
#/calendar from data/calendar.yaml with fiscal-year mapping, role and
to-be filters, month drill-down; #/scenario/<key> storyboard frames with
sample data and review prompts (overlay scenarios/*.json); questionnaire
role filter; hub band for the lenses. Base site gets the same pages with
default personas.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MpkLoLj38QKKBCShEiHR9
</commit_message>
<xml_diff>
--- a/dist/Apptio_Process_Catalog_L0-L2.xlsx
+++ b/dist/Apptio_Process_Catalog_L0-L2.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="L0 Map" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Process Catalog L0-L2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Variants" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="E2E Flow Steps" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="BPMN Diagrams" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Tool Config Reference" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Framework Reference" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Operating Calendar" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Changelog" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="L0 Map" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Process Catalog L0-L2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variants" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E2E Flow Steps" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BPMN Diagrams" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tool Config Reference" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Framework Reference" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Calendar" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changelog" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'L0 Map'!$A$1:$H$1</definedName>

</xml_diff>